<commit_message>
Updated v18 to handle lifestages that are pupa and nymph - long form did not have isotope collection type, and  merucy didn't have choices this has been fixed
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v18.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v18.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D85611B7-4F96-A945-B258-1AE02DE3C963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0863B693-A905-4849-9C7A-9504CB1D5198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -44083,9 +44083,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE6:AE1000" xr:uid="{9917EF8E-9D15-EA4E-B86B-60B39CF888A1}">
       <formula1>"Parr oxygen bomb, Parr semi-micro oxygen bomb, Phillipson microbomb, Gentry-Weigert bomb, Unknown bomb, Proximate composition, Organic analysis, Wet digestion, Unknown"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M6:M1000" xr:uid="{15E17D1F-987D-C745-9314-52B2C8C66A40}">
-      <formula1>"fry, larva, juvenile, adult "</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V6:V10000" xr:uid="{783A5061-181E-6647-B48C-F16794E29794}">
       <formula1>"belly flap, blood, carcass, cleithra, eye lens, egg, fin, gonad, heart, liver, muscle, otolith, scale, spine, stomach, viscera, whole body, whole body (gonads removed), whole body (stomach removed)"</formula1>
     </dataValidation>
@@ -44095,6 +44092,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T6:T10000" xr:uid="{FE3B4961-9F35-5942-85C0-C97B5B164DB5}">
       <formula1>"Idividual, Composite, Mean, SD, Equation"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M6:M10000" xr:uid="{D77F31B9-1615-2E41-A61E-3373EC534A30}">
+      <formula1>"fry, larva, nymph, pupa, juvenile, adult "</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>